<commit_message>
sample leads for upload added and lead distribution router
</commit_message>
<xml_diff>
--- a/dist/sample-leads.xlsx
+++ b/dist/sample-leads.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GANESH\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GANESH\Desktop\vici_frontend\Vici_Frontend_Production\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>phone_number</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>Forex_expo</t>
+  </si>
+  <si>
+    <t>agent_id</t>
   </si>
 </sst>
 </file>
@@ -87,10 +90,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
@@ -401,7 +405,7 @@
     <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -417,8 +421,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>919452015231</v>
       </c>
@@ -434,8 +441,11 @@
       <c r="E2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="3">
+        <v>8999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>919067869241</v>
       </c>
@@ -451,8 +461,11 @@
       <c r="E3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="3">
+        <v>8999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>919524281833</v>
       </c>
@@ -468,29 +481,32 @@
       <c r="E4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="3">
+        <v>8012</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E13" s="2"/>
     </row>
   </sheetData>

</xml_diff>